<commit_message>
refactor: 目录正交化——projects/<game>/<lang>/ × languages/<code>/
- 项目去语言后缀：nrc-th/nrc-en/nrc-common/wwm → nrc/{th,en,common}/wwm/en，语言维度由目录层级表达
- languages/ 按 code 分文件夹：固定名 attributes.json + eval_notes.md（存在即挂载，删 eval_notes 字段改约定）
- _load_project 锚定 skill 根（修 CWD 依赖坑），项目名=<game>/<lang> 路径式
- adjudications 相对引用 ../nrc-common/ → ../common/；profile name 同步
- xiuxiu 参考残件随用户工作区删除一并移除（非 LQE 项目）

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/PM反馈检查项修改报告.xlsx
+++ b/docs/PM反馈检查项修改报告.xlsx
@@ -594,12 +594,12 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>句尾比对不必用 AI 计数，确定性代码即可：源文以「。！？…」结尾而译文句尾无终止标点（.!?…），或源文无句尾标点而译文擅自添加 → Punctuation Minor。句中句号不做 1:1 数量对账——中英句子合法拆合（一句中文译成两句英文）会大量误报，该部分写入 AI 评估关注点，由 AI 结合语义判断是否漏句。泰语等无句号体系语言由语言属性（languages/th.json：sentence_terminator=none）自动判定不适用，无需逐项目配置。</t>
+          <t>句尾比对不必用 AI 计数，确定性代码即可：源文以「。！？…」结尾而译文句尾无终止标点（.!?…），或源文无句尾标点而译文擅自添加 → Punctuation Minor。句中句号不做 1:1 数量对账——中英句子合法拆合（一句中文译成两句英文）会大量误报，该部分写入 AI 评估关注点，由 AI 结合语义判断是否漏句。泰语等无句号体系语言由语言属性（languages/th/：sentence_terminator=none）自动判定不适用，无需逐项目配置。</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>scripts/lqe_io.py；languages/th.json（属性自动判定）；清单文档</t>
+          <t>scripts/lqe_io.py；languages/th/（属性自动判定）；清单文档</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">

</xml_diff>

<commit_message>
feat: N5-N9 + PM 裁决项全量落码（PM 批准 2026-06-12）
- N5 句尾终止标点 / N6 中文数字+量词（含泰文数字数词）/ N7 词重复 / N8 词内大小写 / N9 半角成对标点
- #3 通用标签数量对账（<>/[] 兜底）+ custom type=count_match 项目精配架构
- #7 术语全大写缩写大小写校验（仅缩写、Company style Major，按 PM 裁决收窄）
- #10 省略号文件内混用检查（PM 改不混用方案，零项目配置）
- 语言属性推导落地：th 自动关 N5/N7/N8/#7；numerals=thai 启用泰文数词
- term_map 改 4 元组保留原 case；术语缺译报错显示原始大小写
- 测试 20/20 + th 关断 + count_match 全过；SKILL.md/languages README/清单(md+xlsx)/PM 报告状态同步

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/PM反馈检查项修改报告.xlsx
+++ b/docs/PM反馈检查项修改报告.xlsx
@@ -523,14 +523,14 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>状态：全部待批准；批准后落码，并同步《质量检查项清单》（md 与 xlsx）</t>
+          <t>状态：PM 已批准（2026-06-12）并全部实施——N5–N9、#3 通用标签对账+custom count_match、#7 缩写大小写（Major）、#10 省略号混用检查；#2 泰语数词已纳入；#5 的 20 字分档随 N2 实施线记录</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>需要 PM 动作的共 5 条（#2/#3/#5/#7/#10，见最后一列）；其余 5 条无需提供任何材料，批准即可实施</t>
+          <t>PM 反馈已全部消化：#2 仅带量词触发+泰语纳入；#3 转通用标签模式集兜底（无需再提供样例，特殊格式后续遇到再精配）；#5 阈值 20 字；#7 仅全大写缩写、判严重；#10 转为文件内不混用检查</t>
         </is>
       </c>
     </row>

</xml_diff>